<commit_message>
fix: correct ddl statements and xlsx file for proper database population
</commit_message>
<xml_diff>
--- a/sql/hotelchains.xlsx
+++ b/sql/hotelchains.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniela Bordeianu\Uni\CSI2132\room4u\sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBDBB87-7EA1-46D8-A651-5477A4764003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C514FA6-EE96-4F5B-BDE3-2695A8ABA159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7AC72208-6A4A-45CD-80D5-6B3DF0A8B70B}"/>
+    <workbookView xWindow="2520" yWindow="1104" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="6" xr2:uid="{7AC72208-6A4A-45CD-80D5-6B3DF0A8B70B}"/>
   </bookViews>
   <sheets>
     <sheet name="hotel_chain" sheetId="1" r:id="rId1"/>
@@ -885,9 +885,6 @@
     <t>royal</t>
   </si>
   <si>
-    <t>presidential</t>
-  </si>
-  <si>
     <t>view_of_room</t>
   </si>
   <si>
@@ -1279,6 +1276,9 @@
   </si>
   <si>
     <t>Co-op Student</t>
+  </si>
+  <si>
+    <t>penthouse</t>
   </si>
 </sst>
 </file>
@@ -1286,10 +1286,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="168" formatCode="00000"/>
-    <numFmt numFmtId="169" formatCode="000000000"/>
-    <numFmt numFmtId="170" formatCode="0000000000"/>
-    <numFmt numFmtId="173" formatCode="yyyy/mm/dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="00000"/>
+    <numFmt numFmtId="165" formatCode="000000000"/>
+    <numFmt numFmtId="166" formatCode="0000000000"/>
+    <numFmt numFmtId="167" formatCode="yyyy/mm/dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -1331,11 +1331,11 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1723,7 +1723,7 @@
         <v>20814</v>
       </c>
       <c r="H2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1749,7 +1749,7 @@
         <v>22102</v>
       </c>
       <c r="H3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1775,7 +1775,7 @@
         <v>60606</v>
       </c>
       <c r="H4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1801,7 +1801,7 @@
         <v>7054</v>
       </c>
       <c r="H5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1827,7 +1827,7 @@
         <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -1849,7 +1849,7 @@
         <v>266</v>
       </c>
       <c r="C1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1860,7 +1860,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1871,7 +1871,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1882,7 +1882,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1893,7 +1893,7 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1904,7 +1904,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1915,7 +1915,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1926,7 +1926,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1937,7 +1937,7 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1948,7 +1948,7 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1959,7 +1959,7 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1970,7 +1970,7 @@
         <v>3</v>
       </c>
       <c r="C12" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1981,7 +1981,7 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1992,7 +1992,7 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -2003,7 +2003,7 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -2014,7 +2014,7 @@
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -2025,7 +2025,7 @@
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -2036,7 +2036,7 @@
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -2047,7 +2047,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2065,16 +2065,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B1" t="s">
         <v>295</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>296</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>297</v>
-      </c>
-      <c r="D1" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2321,10 +2321,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2332,7 +2332,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -2340,7 +2340,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -2348,7 +2348,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -2356,7 +2356,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -2364,7 +2364,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -2372,7 +2372,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -2380,7 +2380,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -2388,7 +2388,7 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -2396,7 +2396,7 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -2404,7 +2404,7 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -2412,7 +2412,7 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -2420,7 +2420,7 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -2428,7 +2428,7 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -2446,13 +2446,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C1" t="s">
         <v>311</v>
-      </c>
-      <c r="C1" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -2460,7 +2460,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C2" s="5">
         <v>46044.5</v>
@@ -2471,7 +2471,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C3" s="5">
         <v>45691.708668981482</v>
@@ -2482,7 +2482,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C4" s="5">
         <v>45997.916666666664</v>
@@ -2493,7 +2493,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C5" s="5">
         <v>46082.417303240742</v>
@@ -2504,7 +2504,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C6" s="5">
         <v>45792.417013888888</v>
@@ -2515,7 +2515,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C7" s="5">
         <v>46026.440972222219</v>
@@ -2536,13 +2536,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B1" t="s">
+        <v>315</v>
+      </c>
+      <c r="C1" t="s">
         <v>316</v>
-      </c>
-      <c r="C1" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -2670,19 +2670,19 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B1" t="s">
         <v>318</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>319</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E1" t="s">
         <v>320</v>
-      </c>
-      <c r="D1" t="s">
-        <v>322</v>
-      </c>
-      <c r="E1" t="s">
-        <v>321</v>
       </c>
       <c r="F1" t="s">
         <v>11</v>
@@ -2708,22 +2708,22 @@
         <v>124567890</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2" t="s">
+        <v>324</v>
+      </c>
+      <c r="D2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E2" t="s">
         <v>325</v>
-      </c>
-      <c r="D2" t="s">
-        <v>331</v>
-      </c>
-      <c r="E2" t="s">
-        <v>326</v>
       </c>
       <c r="F2">
         <v>125</v>
       </c>
       <c r="G2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H2" t="s">
         <v>104</v>
@@ -2735,7 +2735,7 @@
         <v>12345</v>
       </c>
       <c r="K2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -2743,19 +2743,19 @@
         <v>245667189</v>
       </c>
       <c r="B3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C3" t="s">
+        <v>328</v>
+      </c>
+      <c r="E3" t="s">
         <v>329</v>
-      </c>
-      <c r="E3" t="s">
-        <v>330</v>
       </c>
       <c r="F3">
         <v>99</v>
       </c>
       <c r="G3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H3" t="s">
         <v>79</v>
@@ -2767,7 +2767,7 @@
         <v>67897</v>
       </c>
       <c r="K3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -2775,22 +2775,22 @@
         <v>565224156</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C4" t="s">
+        <v>333</v>
+      </c>
+      <c r="D4" t="s">
         <v>334</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>335</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="s">
         <v>336</v>
-      </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="G4" t="s">
-        <v>337</v>
       </c>
       <c r="H4" t="s">
         <v>139</v>
@@ -2802,7 +2802,7 @@
         <v>78755</v>
       </c>
       <c r="K4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -2810,19 +2810,19 @@
         <v>123456789</v>
       </c>
       <c r="B5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F5">
         <v>678</v>
       </c>
       <c r="G5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H5" t="s">
         <v>104</v>
@@ -2834,7 +2834,7 @@
         <v>54552</v>
       </c>
       <c r="K5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -2842,31 +2842,31 @@
         <v>789123428</v>
       </c>
       <c r="B6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F6">
         <v>178</v>
       </c>
       <c r="G6" t="s">
+        <v>341</v>
+      </c>
+      <c r="H6" t="s">
         <v>342</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>343</v>
-      </c>
-      <c r="I6" t="s">
-        <v>344</v>
       </c>
       <c r="J6">
         <v>88981</v>
       </c>
       <c r="K6" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -2874,34 +2874,34 @@
         <v>124567890</v>
       </c>
       <c r="B7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C7" t="s">
+        <v>344</v>
+      </c>
+      <c r="D7" t="s">
         <v>345</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>346</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" t="s">
         <v>347</v>
       </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>348</v>
       </c>
-      <c r="H7" t="s">
-        <v>349</v>
-      </c>
       <c r="I7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="J7">
         <v>87981</v>
       </c>
       <c r="K7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -2909,34 +2909,34 @@
         <v>245667189</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C8" t="s">
+        <v>349</v>
+      </c>
+      <c r="D8" t="s">
+        <v>351</v>
+      </c>
+      <c r="E8" t="s">
         <v>350</v>
-      </c>
-      <c r="D8" t="s">
-        <v>352</v>
-      </c>
-      <c r="E8" t="s">
-        <v>351</v>
       </c>
       <c r="F8">
         <v>89</v>
       </c>
       <c r="G8" t="s">
+        <v>352</v>
+      </c>
+      <c r="H8" t="s">
+        <v>354</v>
+      </c>
+      <c r="I8" t="s">
         <v>353</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>355</v>
       </c>
-      <c r="I8" t="s">
-        <v>354</v>
-      </c>
-      <c r="J8" t="s">
-        <v>356</v>
-      </c>
       <c r="K8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -2944,19 +2944,19 @@
         <v>565224156</v>
       </c>
       <c r="B9" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C9" t="s">
+        <v>356</v>
+      </c>
+      <c r="E9" t="s">
         <v>357</v>
-      </c>
-      <c r="E9" t="s">
-        <v>358</v>
       </c>
       <c r="F9">
         <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="H9" t="s">
         <v>27</v>
@@ -2965,10 +2965,10 @@
         <v>28</v>
       </c>
       <c r="J9" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="K9" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -2976,34 +2976,34 @@
         <v>786124431</v>
       </c>
       <c r="B10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D10" t="s">
         <v>362</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>363</v>
-      </c>
-      <c r="E10" t="s">
-        <v>364</v>
       </c>
       <c r="F10">
         <v>554</v>
       </c>
       <c r="G10" t="s">
+        <v>364</v>
+      </c>
+      <c r="H10" t="s">
+        <v>366</v>
+      </c>
+      <c r="I10" t="s">
         <v>365</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
         <v>367</v>
       </c>
-      <c r="I10" t="s">
-        <v>366</v>
-      </c>
-      <c r="J10" t="s">
-        <v>368</v>
-      </c>
       <c r="K10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -3011,22 +3011,22 @@
         <v>662112345</v>
       </c>
       <c r="B11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C11" t="s">
+        <v>368</v>
+      </c>
+      <c r="D11" t="s">
         <v>369</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>370</v>
-      </c>
-      <c r="E11" t="s">
-        <v>371</v>
       </c>
       <c r="F11">
         <v>99</v>
       </c>
       <c r="G11" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="H11" t="s">
         <v>75</v>
@@ -3035,10 +3035,10 @@
         <v>76</v>
       </c>
       <c r="J11" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="K11" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -3046,31 +3046,31 @@
         <v>223761213</v>
       </c>
       <c r="B12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E12" t="s">
         <v>389</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12" t="s">
         <v>390</v>
       </c>
-      <c r="F12">
-        <v>2</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>391</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
+        <v>353</v>
+      </c>
+      <c r="J12" t="s">
         <v>392</v>
       </c>
-      <c r="I12" t="s">
-        <v>354</v>
-      </c>
-      <c r="J12" t="s">
-        <v>393</v>
-      </c>
       <c r="K12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -3078,34 +3078,34 @@
         <v>111676789</v>
       </c>
       <c r="B13" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C13" t="s">
+        <v>393</v>
+      </c>
+      <c r="D13" t="s">
         <v>394</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>395</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13" t="s">
         <v>396</v>
       </c>
-      <c r="F13">
-        <v>4</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>397</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
+        <v>353</v>
+      </c>
+      <c r="J13" t="s">
         <v>398</v>
       </c>
-      <c r="I13" t="s">
-        <v>354</v>
-      </c>
-      <c r="J13" t="s">
-        <v>399</v>
-      </c>
       <c r="K13" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -3113,34 +3113,34 @@
         <v>222676789</v>
       </c>
       <c r="B14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C14" t="s">
+        <v>399</v>
+      </c>
+      <c r="D14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E14" t="s">
         <v>400</v>
-      </c>
-      <c r="D14" t="s">
-        <v>402</v>
-      </c>
-      <c r="E14" t="s">
-        <v>401</v>
       </c>
       <c r="F14">
         <v>8</v>
       </c>
       <c r="G14" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H14" t="s">
         <v>146</v>
       </c>
       <c r="I14" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J14" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="K14" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -3158,10 +3158,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B1" t="s">
         <v>318</v>
-      </c>
-      <c r="B1" t="s">
-        <v>319</v>
       </c>
       <c r="C1" t="s">
         <v>30</v>
@@ -3172,7 +3172,7 @@
         <v>124567890</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2">
         <v>4</v>
@@ -3183,7 +3183,7 @@
         <v>245667189</v>
       </c>
       <c r="B3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -3191,7 +3191,7 @@
         <v>565224156</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C4">
         <v>44</v>
@@ -3202,7 +3202,7 @@
         <v>786124431</v>
       </c>
       <c r="B5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C5">
         <v>44</v>
@@ -3213,7 +3213,7 @@
         <v>662112345</v>
       </c>
       <c r="B6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C6">
         <v>23</v>
@@ -3224,7 +3224,7 @@
         <v>223761213</v>
       </c>
       <c r="B7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -3235,7 +3235,7 @@
         <v>111676789</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -3243,7 +3243,7 @@
         <v>222676789</v>
       </c>
       <c r="B9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -3261,13 +3261,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B1" t="s">
         <v>318</v>
       </c>
-      <c r="B1" t="s">
-        <v>319</v>
-      </c>
       <c r="C1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -3275,10 +3275,10 @@
         <v>124567890</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3286,10 +3286,10 @@
         <v>245667189</v>
       </c>
       <c r="B3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -3297,10 +3297,10 @@
         <v>565224156</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -3308,10 +3308,10 @@
         <v>786124431</v>
       </c>
       <c r="B5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -3319,10 +3319,10 @@
         <v>662112345</v>
       </c>
       <c r="B6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -3330,10 +3330,10 @@
         <v>662112345</v>
       </c>
       <c r="B7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -3341,10 +3341,10 @@
         <v>662112345</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -3352,10 +3352,10 @@
         <v>565224156</v>
       </c>
       <c r="B9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C9" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -3363,10 +3363,10 @@
         <v>565224156</v>
       </c>
       <c r="B10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -3374,10 +3374,10 @@
         <v>786124431</v>
       </c>
       <c r="B11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -3385,10 +3385,10 @@
         <v>662112345</v>
       </c>
       <c r="B12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C12" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -3396,10 +3396,10 @@
         <v>223761213</v>
       </c>
       <c r="B13" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -3407,10 +3407,10 @@
         <v>111676789</v>
       </c>
       <c r="B14" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -3418,10 +3418,10 @@
         <v>222676789</v>
       </c>
       <c r="B15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C15" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -3440,13 +3440,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B1" t="s">
         <v>318</v>
       </c>
-      <c r="B1" t="s">
-        <v>319</v>
-      </c>
       <c r="C1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -3454,7 +3454,7 @@
         <v>123456789</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2" s="5">
         <v>45323.506643518522</v>
@@ -3465,7 +3465,7 @@
         <v>789123428</v>
       </c>
       <c r="B3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C3" s="5">
         <v>45413.961909722224</v>
@@ -3476,7 +3476,7 @@
         <v>124567890</v>
       </c>
       <c r="B4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C4" s="5">
         <v>45484.481990740744</v>
@@ -3487,7 +3487,7 @@
         <v>245667189</v>
       </c>
       <c r="B5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C5" s="5">
         <v>45272.008472222224</v>
@@ -3498,7 +3498,7 @@
         <v>565224156</v>
       </c>
       <c r="B6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C6" s="5">
         <v>45173.418564814812</v>
@@ -3516,7 +3516,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B1" t="s">
         <v>30</v>
@@ -3717,7 +3717,7 @@
         <v>77</v>
       </c>
       <c r="J2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -3749,7 +3749,7 @@
         <v>10022</v>
       </c>
       <c r="J3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -3781,7 +3781,7 @@
         <v>28202</v>
       </c>
       <c r="J4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -3813,7 +3813,7 @@
         <v>33140</v>
       </c>
       <c r="J5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -3845,7 +3845,7 @@
         <v>10003</v>
       </c>
       <c r="J6" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -3877,7 +3877,7 @@
         <v>96815</v>
       </c>
       <c r="J7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -3909,7 +3909,7 @@
         <v>2114</v>
       </c>
       <c r="J8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -3941,7 +3941,7 @@
         <v>92802</v>
       </c>
       <c r="J9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -3973,7 +3973,7 @@
         <v>10022</v>
       </c>
       <c r="J10" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -4005,7 +4005,7 @@
         <v>85016</v>
       </c>
       <c r="J11" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -4037,7 +4037,7 @@
         <v>10282</v>
       </c>
       <c r="J12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -4069,7 +4069,7 @@
         <v>32821</v>
       </c>
       <c r="J13" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -4101,7 +4101,7 @@
         <v>10019</v>
       </c>
       <c r="J14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -4133,7 +4133,7 @@
         <v>108</v>
       </c>
       <c r="J15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -4165,7 +4165,7 @@
         <v>110</v>
       </c>
       <c r="J16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -4197,7 +4197,7 @@
         <v>112</v>
       </c>
       <c r="J17" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -4229,7 +4229,7 @@
         <v>10036</v>
       </c>
       <c r="J18" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
@@ -4261,7 +4261,7 @@
         <v>10019</v>
       </c>
       <c r="J19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -4293,7 +4293,7 @@
         <v>116</v>
       </c>
       <c r="J20" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
@@ -4325,7 +4325,7 @@
         <v>118</v>
       </c>
       <c r="J21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -4357,7 +4357,7 @@
         <v>120</v>
       </c>
       <c r="J22" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
@@ -4389,7 +4389,7 @@
         <v>122</v>
       </c>
       <c r="J23" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
@@ -4421,7 +4421,7 @@
         <v>32819</v>
       </c>
       <c r="J24" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
@@ -4453,7 +4453,7 @@
         <v>10036</v>
       </c>
       <c r="J25" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
@@ -4485,7 +4485,7 @@
         <v>94087</v>
       </c>
       <c r="J26" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
@@ -4517,7 +4517,7 @@
         <v>130</v>
       </c>
       <c r="J27" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -4549,7 +4549,7 @@
         <v>33767</v>
       </c>
       <c r="J28" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -4581,7 +4581,7 @@
         <v>8205</v>
       </c>
       <c r="J29" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
@@ -4613,7 +4613,7 @@
         <v>80903</v>
       </c>
       <c r="J30" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
@@ -4645,7 +4645,7 @@
         <v>94080</v>
       </c>
       <c r="J31" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
@@ -4677,7 +4677,7 @@
         <v>11101</v>
       </c>
       <c r="J32" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
@@ -4709,7 +4709,7 @@
         <v>34747</v>
       </c>
       <c r="J33" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
@@ -4741,7 +4741,7 @@
         <v>32819</v>
       </c>
       <c r="J34" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
@@ -4773,7 +4773,7 @@
         <v>40202</v>
       </c>
       <c r="J35" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
@@ -4805,7 +4805,7 @@
         <v>94123</v>
       </c>
       <c r="J36" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
@@ -4837,7 +4837,7 @@
         <v>150</v>
       </c>
       <c r="J37" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
@@ -4869,7 +4869,7 @@
         <v>158</v>
       </c>
       <c r="J38" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
@@ -4901,7 +4901,7 @@
         <v>160</v>
       </c>
       <c r="J39" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
@@ -4933,7 +4933,7 @@
         <v>163</v>
       </c>
       <c r="J40" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
@@ -4965,7 +4965,7 @@
         <v>167</v>
       </c>
       <c r="J41" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
@@ -4997,7 +4997,7 @@
         <v>170</v>
       </c>
       <c r="J42" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
@@ -5029,7 +5029,7 @@
         <v>172</v>
       </c>
       <c r="J43" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
@@ -5061,7 +5061,7 @@
         <v>174</v>
       </c>
       <c r="J44" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
@@ -5093,7 +5093,7 @@
         <v>176</v>
       </c>
       <c r="J45" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -5111,13 +5111,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C1" t="s">
         <v>318</v>
-      </c>
-      <c r="C1" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -5128,7 +5128,7 @@
         <v>123456789</v>
       </c>
       <c r="C2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -5139,7 +5139,7 @@
         <v>789123428</v>
       </c>
       <c r="C3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -5150,7 +5150,7 @@
         <v>124567890</v>
       </c>
       <c r="C4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -5161,7 +5161,7 @@
         <v>245667189</v>
       </c>
       <c r="C5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -5172,7 +5172,7 @@
         <v>565224156</v>
       </c>
       <c r="C6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -5183,7 +5183,7 @@
         <v>124567890</v>
       </c>
       <c r="C7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -5194,7 +5194,7 @@
         <v>123456789</v>
       </c>
       <c r="C8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -5205,7 +5205,7 @@
         <v>789123428</v>
       </c>
       <c r="C9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -5216,7 +5216,7 @@
         <v>245667189</v>
       </c>
       <c r="C10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -5227,7 +5227,7 @@
         <v>565224156</v>
       </c>
       <c r="C11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -5238,7 +5238,7 @@
         <v>124567890</v>
       </c>
       <c r="C12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -5256,10 +5256,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B1" t="s">
         <v>318</v>
-      </c>
-      <c r="B1" t="s">
-        <v>319</v>
       </c>
       <c r="C1" t="s">
         <v>30</v>
@@ -5270,7 +5270,7 @@
         <v>124567890</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2">
         <v>4</v>
@@ -5281,7 +5281,7 @@
         <v>245667189</v>
       </c>
       <c r="B3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -5292,7 +5292,7 @@
         <v>565224156</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C4">
         <v>44</v>
@@ -5303,7 +5303,7 @@
         <v>786124431</v>
       </c>
       <c r="B5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C5">
         <v>44</v>
@@ -5314,7 +5314,7 @@
         <v>662112345</v>
       </c>
       <c r="B6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C6">
         <v>23</v>
@@ -5325,7 +5325,7 @@
         <v>223761213</v>
       </c>
       <c r="B7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -5336,7 +5336,7 @@
         <v>111676789</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -5347,7 +5347,7 @@
         <v>222676789</v>
       </c>
       <c r="B9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -5369,16 +5369,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B1" t="s">
         <v>384</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>385</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>386</v>
-      </c>
-      <c r="D1" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -5386,13 +5386,13 @@
         <v>565224156</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2" s="3">
         <v>786124431</v>
       </c>
       <c r="D2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -5400,7 +5400,7 @@
         <v>786124431</v>
       </c>
       <c r="B3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -5408,7 +5408,7 @@
         <v>124567890</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -5416,13 +5416,13 @@
         <v>245667189</v>
       </c>
       <c r="B5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C5">
         <v>223761213</v>
       </c>
       <c r="D5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -5430,7 +5430,7 @@
         <v>662112345</v>
       </c>
       <c r="B6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -5438,7 +5438,7 @@
         <v>223761213</v>
       </c>
       <c r="B7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -5446,13 +5446,13 @@
         <v>111676789</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C8">
         <v>223761213</v>
       </c>
       <c r="D8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -5460,13 +5460,13 @@
         <v>222676789</v>
       </c>
       <c r="B9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C9">
         <v>223761213</v>
       </c>
       <c r="D9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -5484,13 +5484,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B1" t="s">
         <v>318</v>
       </c>
-      <c r="B1" t="s">
-        <v>319</v>
-      </c>
       <c r="C1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -5498,7 +5498,7 @@
         <v>124567890</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -5509,7 +5509,7 @@
         <v>245667189</v>
       </c>
       <c r="B3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -5520,7 +5520,7 @@
         <v>565224156</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -5531,7 +5531,7 @@
         <v>786124431</v>
       </c>
       <c r="B5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -5542,7 +5542,7 @@
         <v>662112345</v>
       </c>
       <c r="B6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -5553,7 +5553,7 @@
         <v>223761213</v>
       </c>
       <c r="B7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -5564,7 +5564,7 @@
         <v>111676789</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -5575,7 +5575,7 @@
         <v>222676789</v>
       </c>
       <c r="B9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C9">
         <v>8</v>
@@ -5586,7 +5586,7 @@
         <v>223761213</v>
       </c>
       <c r="B10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -5597,7 +5597,7 @@
         <v>111676789</v>
       </c>
       <c r="B11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -5608,7 +5608,7 @@
         <v>222676789</v>
       </c>
       <c r="B12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C12">
         <v>11</v>
@@ -7479,7 +7479,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="D6" t="s">
         <v>274</v>
@@ -7564,10 +7564,10 @@
         <v>5</v>
       </c>
       <c r="C11">
-        <v>50000</v>
+        <v>9000</v>
       </c>
       <c r="D11" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -7649,7 +7649,7 @@
         <v>5</v>
       </c>
       <c r="C16">
-        <v>10000</v>
+        <v>9000</v>
       </c>
       <c r="D16" t="s">
         <v>274</v>
@@ -7734,10 +7734,10 @@
         <v>5</v>
       </c>
       <c r="C21">
-        <v>10000</v>
+        <v>9090</v>
       </c>
       <c r="D21" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -7819,7 +7819,7 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D26" t="s">
         <v>274</v>
@@ -7904,10 +7904,10 @@
         <v>5</v>
       </c>
       <c r="C31">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D31" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -7989,7 +7989,7 @@
         <v>5</v>
       </c>
       <c r="C36">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D36" t="s">
         <v>274</v>
@@ -8077,7 +8077,7 @@
         <v>1500</v>
       </c>
       <c r="D41" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -8247,7 +8247,7 @@
         <v>1500</v>
       </c>
       <c r="D51" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
@@ -8329,7 +8329,7 @@
         <v>5</v>
       </c>
       <c r="C56">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D56" t="s">
         <v>274</v>
@@ -8414,10 +8414,10 @@
         <v>5</v>
       </c>
       <c r="C61">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D61" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E61" t="b">
         <v>1</v>
@@ -8465,7 +8465,7 @@
         <v>3</v>
       </c>
       <c r="C64">
-        <v>15500</v>
+        <v>1550</v>
       </c>
       <c r="D64" t="s">
         <v>272</v>
@@ -8499,7 +8499,7 @@
         <v>5</v>
       </c>
       <c r="C66">
-        <v>25670</v>
+        <v>5670</v>
       </c>
       <c r="D66" t="s">
         <v>274</v>
@@ -8550,7 +8550,7 @@
         <v>3</v>
       </c>
       <c r="C69">
-        <v>15500</v>
+        <v>1550</v>
       </c>
       <c r="D69" t="s">
         <v>272</v>
@@ -8584,10 +8584,10 @@
         <v>5</v>
       </c>
       <c r="C71">
-        <v>25670</v>
+        <v>2560</v>
       </c>
       <c r="D71" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -8635,7 +8635,7 @@
         <v>3</v>
       </c>
       <c r="C74">
-        <v>15500</v>
+        <v>5500</v>
       </c>
       <c r="D74" t="s">
         <v>272</v>
@@ -8669,7 +8669,7 @@
         <v>5</v>
       </c>
       <c r="C76">
-        <v>25670</v>
+        <v>2567</v>
       </c>
       <c r="D76" t="s">
         <v>274</v>
@@ -8720,7 +8720,7 @@
         <v>3</v>
       </c>
       <c r="C79">
-        <v>15500</v>
+        <v>5500</v>
       </c>
       <c r="D79" t="s">
         <v>272</v>
@@ -8754,10 +8754,10 @@
         <v>5</v>
       </c>
       <c r="C81">
-        <v>25670</v>
+        <v>5670</v>
       </c>
       <c r="D81" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E81" t="b">
         <v>1</v>
@@ -8805,7 +8805,7 @@
         <v>3</v>
       </c>
       <c r="C84">
-        <v>15500</v>
+        <v>5500</v>
       </c>
       <c r="D84" t="s">
         <v>272</v>
@@ -8839,7 +8839,7 @@
         <v>5</v>
       </c>
       <c r="C86">
-        <v>25670</v>
+        <v>5670</v>
       </c>
       <c r="D86" t="s">
         <v>274</v>
@@ -8924,10 +8924,10 @@
         <v>5</v>
       </c>
       <c r="C91">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D91" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E91" t="b">
         <v>1</v>
@@ -9009,7 +9009,7 @@
         <v>5</v>
       </c>
       <c r="C96">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D96" t="s">
         <v>274</v>
@@ -9094,10 +9094,10 @@
         <v>5</v>
       </c>
       <c r="C101">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D101" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -9179,7 +9179,7 @@
         <v>5</v>
       </c>
       <c r="C106">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D106" t="s">
         <v>274</v>
@@ -9264,10 +9264,10 @@
         <v>5</v>
       </c>
       <c r="C111">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D111" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E111" t="b">
         <v>1</v>
@@ -9349,7 +9349,7 @@
         <v>5</v>
       </c>
       <c r="C116">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D116" t="s">
         <v>274</v>
@@ -9434,10 +9434,10 @@
         <v>5</v>
       </c>
       <c r="C121">
-        <v>10000</v>
+        <v>9000</v>
       </c>
       <c r="D121" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E121" t="b">
         <v>1</v>
@@ -9519,7 +9519,7 @@
         <v>5</v>
       </c>
       <c r="C126">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="D126" t="s">
         <v>274</v>
@@ -9604,10 +9604,10 @@
         <v>5</v>
       </c>
       <c r="C131">
-        <v>10000</v>
+        <v>7000</v>
       </c>
       <c r="D131" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -9689,7 +9689,7 @@
         <v>5</v>
       </c>
       <c r="C136">
-        <v>10000</v>
+        <v>9000</v>
       </c>
       <c r="D136" t="s">
         <v>274</v>
@@ -9774,10 +9774,10 @@
         <v>5</v>
       </c>
       <c r="C141">
-        <v>10000</v>
+        <v>8750</v>
       </c>
       <c r="D141" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E141" t="b">
         <v>1</v>
@@ -9944,10 +9944,10 @@
         <v>5</v>
       </c>
       <c r="C151">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D151" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E151" t="b">
         <v>1</v>
@@ -10029,7 +10029,7 @@
         <v>5</v>
       </c>
       <c r="C156">
-        <v>50000</v>
+        <v>9000</v>
       </c>
       <c r="D156" t="s">
         <v>274</v>
@@ -10114,10 +10114,10 @@
         <v>5</v>
       </c>
       <c r="C161">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D161" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -10199,7 +10199,7 @@
         <v>5</v>
       </c>
       <c r="C166">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D166" t="s">
         <v>274</v>
@@ -10284,10 +10284,10 @@
         <v>5</v>
       </c>
       <c r="C171">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D171" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E171" t="b">
         <v>1</v>
@@ -10369,7 +10369,7 @@
         <v>5</v>
       </c>
       <c r="C176">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D176" t="s">
         <v>274</v>
@@ -10454,10 +10454,10 @@
         <v>5</v>
       </c>
       <c r="C181">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D181" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E181" t="b">
         <v>1</v>
@@ -10539,7 +10539,7 @@
         <v>5</v>
       </c>
       <c r="C186">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D186" t="s">
         <v>274</v>
@@ -10624,10 +10624,10 @@
         <v>5</v>
       </c>
       <c r="C191">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D191" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -10709,7 +10709,7 @@
         <v>5</v>
       </c>
       <c r="C196">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="D196" t="s">
         <v>274</v>
@@ -10797,7 +10797,7 @@
         <v>1500</v>
       </c>
       <c r="D201" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E201" t="b">
         <v>1</v>
@@ -10967,7 +10967,7 @@
         <v>1500</v>
       </c>
       <c r="D211" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E211" t="b">
         <v>1</v>
@@ -11137,7 +11137,7 @@
         <v>1500</v>
       </c>
       <c r="D221" t="s">
-        <v>275</v>
+        <v>406</v>
       </c>
       <c r="E221" t="b">
         <v>0</v>
@@ -11161,7 +11161,7 @@
         <v>266</v>
       </c>
       <c r="C1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -11172,7 +11172,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -11183,7 +11183,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -11194,7 +11194,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -11205,7 +11205,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -11216,7 +11216,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -11227,7 +11227,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -11238,7 +11238,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -11249,7 +11249,7 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -11260,7 +11260,7 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -11271,7 +11271,7 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -11282,7 +11282,7 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -11293,7 +11293,7 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -11304,7 +11304,7 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -11315,7 +11315,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -11326,7 +11326,7 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -11337,7 +11337,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -11348,7 +11348,7 @@
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -11359,7 +11359,7 @@
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -11370,7 +11370,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -11381,7 +11381,7 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -11392,7 +11392,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -11403,7 +11403,7 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -11414,7 +11414,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -11425,7 +11425,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -11436,7 +11436,7 @@
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -11447,7 +11447,7 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -11458,7 +11458,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -11469,7 +11469,7 @@
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -11480,7 +11480,7 @@
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -11491,7 +11491,7 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -11502,7 +11502,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -11513,7 +11513,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -11524,7 +11524,7 @@
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -11535,7 +11535,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -11546,7 +11546,7 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -11557,7 +11557,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -11568,7 +11568,7 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -11579,7 +11579,7 @@
         <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -11590,7 +11590,7 @@
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -11601,7 +11601,7 @@
         <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -11612,7 +11612,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -11623,7 +11623,7 @@
         <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -11634,7 +11634,7 @@
         <v>3</v>
       </c>
       <c r="C44" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -11645,7 +11645,7 @@
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -11656,7 +11656,7 @@
         <v>5</v>
       </c>
       <c r="C46" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -11667,7 +11667,7 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -11678,7 +11678,7 @@
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -11689,7 +11689,7 @@
         <v>3</v>
       </c>
       <c r="C49" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -11700,7 +11700,7 @@
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -11711,7 +11711,7 @@
         <v>5</v>
       </c>
       <c r="C51" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -11722,7 +11722,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -11733,7 +11733,7 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -11744,7 +11744,7 @@
         <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -11755,7 +11755,7 @@
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -11766,7 +11766,7 @@
         <v>5</v>
       </c>
       <c r="C56" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -11777,7 +11777,7 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -11788,7 +11788,7 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -11799,7 +11799,7 @@
         <v>3</v>
       </c>
       <c r="C59" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -11810,7 +11810,7 @@
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -11821,7 +11821,7 @@
         <v>5</v>
       </c>
       <c r="C61" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -11832,7 +11832,7 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -11843,7 +11843,7 @@
         <v>2</v>
       </c>
       <c r="C63" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -11854,7 +11854,7 @@
         <v>3</v>
       </c>
       <c r="C64" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
@@ -11865,7 +11865,7 @@
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
@@ -11876,7 +11876,7 @@
         <v>5</v>
       </c>
       <c r="C66" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -11887,7 +11887,7 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -11898,7 +11898,7 @@
         <v>2</v>
       </c>
       <c r="C68" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -11909,7 +11909,7 @@
         <v>3</v>
       </c>
       <c r="C69" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
@@ -11920,7 +11920,7 @@
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -11931,7 +11931,7 @@
         <v>5</v>
       </c>
       <c r="C71" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -11942,7 +11942,7 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -11953,7 +11953,7 @@
         <v>2</v>
       </c>
       <c r="C73" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
@@ -11964,7 +11964,7 @@
         <v>3</v>
       </c>
       <c r="C74" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
@@ -11975,7 +11975,7 @@
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
@@ -11986,7 +11986,7 @@
         <v>5</v>
       </c>
       <c r="C76" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
@@ -11997,7 +11997,7 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -12008,7 +12008,7 @@
         <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -12019,7 +12019,7 @@
         <v>3</v>
       </c>
       <c r="C79" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -12030,7 +12030,7 @@
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -12041,7 +12041,7 @@
         <v>5</v>
       </c>
       <c r="C81" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -12052,7 +12052,7 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -12063,7 +12063,7 @@
         <v>2</v>
       </c>
       <c r="C83" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
@@ -12074,7 +12074,7 @@
         <v>3</v>
       </c>
       <c r="C84" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
@@ -12085,7 +12085,7 @@
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -12096,7 +12096,7 @@
         <v>5</v>
       </c>
       <c r="C86" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
@@ -12107,7 +12107,7 @@
         <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
@@ -12118,7 +12118,7 @@
         <v>2</v>
       </c>
       <c r="C88" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
@@ -12129,7 +12129,7 @@
         <v>3</v>
       </c>
       <c r="C89" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
@@ -12140,7 +12140,7 @@
         <v>4</v>
       </c>
       <c r="C90" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
@@ -12151,7 +12151,7 @@
         <v>5</v>
       </c>
       <c r="C91" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -12162,7 +12162,7 @@
         <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
@@ -12173,7 +12173,7 @@
         <v>2</v>
       </c>
       <c r="C93" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
@@ -12184,7 +12184,7 @@
         <v>3</v>
       </c>
       <c r="C94" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
@@ -12195,7 +12195,7 @@
         <v>4</v>
       </c>
       <c r="C95" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
@@ -12206,7 +12206,7 @@
         <v>5</v>
       </c>
       <c r="C96" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
@@ -12217,7 +12217,7 @@
         <v>1</v>
       </c>
       <c r="C97" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
@@ -12228,7 +12228,7 @@
         <v>2</v>
       </c>
       <c r="C98" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
@@ -12239,7 +12239,7 @@
         <v>3</v>
       </c>
       <c r="C99" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
@@ -12250,7 +12250,7 @@
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
@@ -12261,7 +12261,7 @@
         <v>5</v>
       </c>
       <c r="C101" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
@@ -12272,7 +12272,7 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
@@ -12283,7 +12283,7 @@
         <v>2</v>
       </c>
       <c r="C103" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
@@ -12294,7 +12294,7 @@
         <v>3</v>
       </c>
       <c r="C104" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
@@ -12305,7 +12305,7 @@
         <v>4</v>
       </c>
       <c r="C105" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
@@ -12316,7 +12316,7 @@
         <v>5</v>
       </c>
       <c r="C106" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
@@ -12327,7 +12327,7 @@
         <v>1</v>
       </c>
       <c r="C107" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
@@ -12338,7 +12338,7 @@
         <v>2</v>
       </c>
       <c r="C108" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
@@ -12349,7 +12349,7 @@
         <v>3</v>
       </c>
       <c r="C109" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
@@ -12360,7 +12360,7 @@
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
@@ -12371,7 +12371,7 @@
         <v>5</v>
       </c>
       <c r="C111" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.3">
@@ -12382,7 +12382,7 @@
         <v>1</v>
       </c>
       <c r="C112" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
@@ -12393,7 +12393,7 @@
         <v>2</v>
       </c>
       <c r="C113" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
@@ -12404,7 +12404,7 @@
         <v>3</v>
       </c>
       <c r="C114" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.3">
@@ -12415,7 +12415,7 @@
         <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.3">
@@ -12426,7 +12426,7 @@
         <v>5</v>
       </c>
       <c r="C116" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.3">
@@ -12437,7 +12437,7 @@
         <v>1</v>
       </c>
       <c r="C117" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
@@ -12448,7 +12448,7 @@
         <v>2</v>
       </c>
       <c r="C118" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
@@ -12459,7 +12459,7 @@
         <v>3</v>
       </c>
       <c r="C119" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
@@ -12470,7 +12470,7 @@
         <v>4</v>
       </c>
       <c r="C120" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
@@ -12481,7 +12481,7 @@
         <v>5</v>
       </c>
       <c r="C121" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
@@ -12492,7 +12492,7 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
@@ -12503,7 +12503,7 @@
         <v>2</v>
       </c>
       <c r="C123" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
@@ -12514,7 +12514,7 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
@@ -12525,7 +12525,7 @@
         <v>4</v>
       </c>
       <c r="C125" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
@@ -12536,7 +12536,7 @@
         <v>5</v>
       </c>
       <c r="C126" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
@@ -12547,7 +12547,7 @@
         <v>1</v>
       </c>
       <c r="C127" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
@@ -12558,7 +12558,7 @@
         <v>2</v>
       </c>
       <c r="C128" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.3">
@@ -12569,7 +12569,7 @@
         <v>3</v>
       </c>
       <c r="C129" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.3">
@@ -12580,7 +12580,7 @@
         <v>4</v>
       </c>
       <c r="C130" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.3">
@@ -12591,7 +12591,7 @@
         <v>5</v>
       </c>
       <c r="C131" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.3">
@@ -12602,7 +12602,7 @@
         <v>1</v>
       </c>
       <c r="C132" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.3">
@@ -12613,7 +12613,7 @@
         <v>2</v>
       </c>
       <c r="C133" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.3">
@@ -12624,7 +12624,7 @@
         <v>3</v>
       </c>
       <c r="C134" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.3">
@@ -12635,7 +12635,7 @@
         <v>4</v>
       </c>
       <c r="C135" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.3">
@@ -12646,7 +12646,7 @@
         <v>5</v>
       </c>
       <c r="C136" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.3">
@@ -12657,7 +12657,7 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.3">
@@ -12668,7 +12668,7 @@
         <v>2</v>
       </c>
       <c r="C138" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.3">
@@ -12679,7 +12679,7 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.3">
@@ -12690,7 +12690,7 @@
         <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.3">
@@ -12701,7 +12701,7 @@
         <v>5</v>
       </c>
       <c r="C141" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.3">
@@ -12712,7 +12712,7 @@
         <v>1</v>
       </c>
       <c r="C142" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.3">
@@ -12723,7 +12723,7 @@
         <v>2</v>
       </c>
       <c r="C143" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.3">
@@ -12734,7 +12734,7 @@
         <v>3</v>
       </c>
       <c r="C144" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
@@ -12745,7 +12745,7 @@
         <v>4</v>
       </c>
       <c r="C145" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.3">
@@ -12756,7 +12756,7 @@
         <v>5</v>
       </c>
       <c r="C146" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.3">
@@ -12767,7 +12767,7 @@
         <v>1</v>
       </c>
       <c r="C147" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.3">
@@ -12778,7 +12778,7 @@
         <v>2</v>
       </c>
       <c r="C148" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.3">
@@ -12789,7 +12789,7 @@
         <v>3</v>
       </c>
       <c r="C149" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.3">
@@ -12800,7 +12800,7 @@
         <v>4</v>
       </c>
       <c r="C150" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.3">
@@ -12811,7 +12811,7 @@
         <v>5</v>
       </c>
       <c r="C151" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.3">
@@ -12822,7 +12822,7 @@
         <v>1</v>
       </c>
       <c r="C152" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.3">
@@ -12833,7 +12833,7 @@
         <v>2</v>
       </c>
       <c r="C153" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.3">
@@ -12844,7 +12844,7 @@
         <v>3</v>
       </c>
       <c r="C154" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
@@ -12855,7 +12855,7 @@
         <v>4</v>
       </c>
       <c r="C155" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.3">
@@ -12866,7 +12866,7 @@
         <v>5</v>
       </c>
       <c r="C156" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.3">
@@ -12877,7 +12877,7 @@
         <v>1</v>
       </c>
       <c r="C157" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.3">
@@ -12888,7 +12888,7 @@
         <v>2</v>
       </c>
       <c r="C158" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.3">
@@ -12899,7 +12899,7 @@
         <v>3</v>
       </c>
       <c r="C159" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.3">
@@ -12910,7 +12910,7 @@
         <v>4</v>
       </c>
       <c r="C160" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.3">
@@ -12921,7 +12921,7 @@
         <v>5</v>
       </c>
       <c r="C161" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.3">
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="C162" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.3">
@@ -12943,7 +12943,7 @@
         <v>2</v>
       </c>
       <c r="C163" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.3">
@@ -12954,7 +12954,7 @@
         <v>3</v>
       </c>
       <c r="C164" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.3">
@@ -12965,7 +12965,7 @@
         <v>4</v>
       </c>
       <c r="C165" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.3">
@@ -12976,7 +12976,7 @@
         <v>5</v>
       </c>
       <c r="C166" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.3">
@@ -12987,7 +12987,7 @@
         <v>1</v>
       </c>
       <c r="C167" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.3">
@@ -12998,7 +12998,7 @@
         <v>2</v>
       </c>
       <c r="C168" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.3">
@@ -13009,7 +13009,7 @@
         <v>3</v>
       </c>
       <c r="C169" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.3">
@@ -13020,7 +13020,7 @@
         <v>4</v>
       </c>
       <c r="C170" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.3">
@@ -13031,7 +13031,7 @@
         <v>5</v>
       </c>
       <c r="C171" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.3">
@@ -13042,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="C172" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.3">
@@ -13053,7 +13053,7 @@
         <v>2</v>
       </c>
       <c r="C173" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.3">
@@ -13064,7 +13064,7 @@
         <v>3</v>
       </c>
       <c r="C174" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.3">
@@ -13075,7 +13075,7 @@
         <v>4</v>
       </c>
       <c r="C175" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.3">
@@ -13086,7 +13086,7 @@
         <v>5</v>
       </c>
       <c r="C176" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.3">
@@ -13097,7 +13097,7 @@
         <v>1</v>
       </c>
       <c r="C177" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.3">
@@ -13108,7 +13108,7 @@
         <v>2</v>
       </c>
       <c r="C178" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.3">
@@ -13119,7 +13119,7 @@
         <v>3</v>
       </c>
       <c r="C179" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.3">
@@ -13130,7 +13130,7 @@
         <v>4</v>
       </c>
       <c r="C180" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.3">
@@ -13141,7 +13141,7 @@
         <v>5</v>
       </c>
       <c r="C181" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.3">
@@ -13152,7 +13152,7 @@
         <v>1</v>
       </c>
       <c r="C182" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.3">
@@ -13163,7 +13163,7 @@
         <v>2</v>
       </c>
       <c r="C183" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.3">
@@ -13174,7 +13174,7 @@
         <v>3</v>
       </c>
       <c r="C184" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.3">
@@ -13185,7 +13185,7 @@
         <v>4</v>
       </c>
       <c r="C185" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.3">
@@ -13196,7 +13196,7 @@
         <v>5</v>
       </c>
       <c r="C186" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.3">
@@ -13207,7 +13207,7 @@
         <v>1</v>
       </c>
       <c r="C187" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.3">
@@ -13218,7 +13218,7 @@
         <v>2</v>
       </c>
       <c r="C188" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.3">
@@ -13229,7 +13229,7 @@
         <v>3</v>
       </c>
       <c r="C189" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.3">
@@ -13240,7 +13240,7 @@
         <v>4</v>
       </c>
       <c r="C190" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.3">
@@ -13251,7 +13251,7 @@
         <v>5</v>
       </c>
       <c r="C191" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.3">
@@ -13262,7 +13262,7 @@
         <v>1</v>
       </c>
       <c r="C192" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.3">
@@ -13273,7 +13273,7 @@
         <v>2</v>
       </c>
       <c r="C193" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.3">
@@ -13284,7 +13284,7 @@
         <v>3</v>
       </c>
       <c r="C194" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.3">
@@ -13295,7 +13295,7 @@
         <v>4</v>
       </c>
       <c r="C195" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.3">
@@ -13306,7 +13306,7 @@
         <v>5</v>
       </c>
       <c r="C196" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.3">
@@ -13317,7 +13317,7 @@
         <v>1</v>
       </c>
       <c r="C197" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.3">
@@ -13328,7 +13328,7 @@
         <v>2</v>
       </c>
       <c r="C198" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.3">
@@ -13339,7 +13339,7 @@
         <v>3</v>
       </c>
       <c r="C199" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.3">
@@ -13350,7 +13350,7 @@
         <v>4</v>
       </c>
       <c r="C200" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.3">
@@ -13361,7 +13361,7 @@
         <v>5</v>
       </c>
       <c r="C201" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.3">
@@ -13372,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="C202" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.3">
@@ -13383,7 +13383,7 @@
         <v>2</v>
       </c>
       <c r="C203" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.3">
@@ -13394,7 +13394,7 @@
         <v>3</v>
       </c>
       <c r="C204" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.3">
@@ -13405,7 +13405,7 @@
         <v>4</v>
       </c>
       <c r="C205" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.3">
@@ -13416,7 +13416,7 @@
         <v>5</v>
       </c>
       <c r="C206" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.3">
@@ -13427,7 +13427,7 @@
         <v>1</v>
       </c>
       <c r="C207" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.3">
@@ -13438,7 +13438,7 @@
         <v>2</v>
       </c>
       <c r="C208" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.3">
@@ -13449,7 +13449,7 @@
         <v>3</v>
       </c>
       <c r="C209" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.3">
@@ -13460,7 +13460,7 @@
         <v>4</v>
       </c>
       <c r="C210" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.3">
@@ -13471,7 +13471,7 @@
         <v>5</v>
       </c>
       <c r="C211" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.3">
@@ -13482,7 +13482,7 @@
         <v>1</v>
       </c>
       <c r="C212" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.3">
@@ -13493,7 +13493,7 @@
         <v>2</v>
       </c>
       <c r="C213" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.3">
@@ -13504,7 +13504,7 @@
         <v>3</v>
       </c>
       <c r="C214" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.3">
@@ -13515,7 +13515,7 @@
         <v>4</v>
       </c>
       <c r="C215" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.3">
@@ -13526,7 +13526,7 @@
         <v>5</v>
       </c>
       <c r="C216" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.3">
@@ -13537,7 +13537,7 @@
         <v>1</v>
       </c>
       <c r="C217" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.3">
@@ -13548,7 +13548,7 @@
         <v>2</v>
       </c>
       <c r="C218" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.3">
@@ -13559,7 +13559,7 @@
         <v>3</v>
       </c>
       <c r="C219" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.3">
@@ -13570,7 +13570,7 @@
         <v>4</v>
       </c>
       <c r="C220" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.3">
@@ -13581,7 +13581,7 @@
         <v>5</v>
       </c>
       <c r="C221" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.3">
@@ -13592,7 +13592,7 @@
         <v>1</v>
       </c>
       <c r="C222" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.3">
@@ -13603,7 +13603,7 @@
         <v>2</v>
       </c>
       <c r="C223" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.3">
@@ -13614,7 +13614,7 @@
         <v>3</v>
       </c>
       <c r="C224" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.3">
@@ -13625,7 +13625,7 @@
         <v>4</v>
       </c>
       <c r="C225" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.3">
@@ -13636,7 +13636,7 @@
         <v>5</v>
       </c>
       <c r="C226" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.3">
@@ -13647,7 +13647,7 @@
         <v>1</v>
       </c>
       <c r="C227" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.3">
@@ -13658,7 +13658,7 @@
         <v>2</v>
       </c>
       <c r="C228" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.3">
@@ -13669,7 +13669,7 @@
         <v>3</v>
       </c>
       <c r="C229" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.3">
@@ -13680,7 +13680,7 @@
         <v>4</v>
       </c>
       <c r="C230" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.3">
@@ -13691,7 +13691,7 @@
         <v>5</v>
       </c>
       <c r="C231" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.3">
@@ -13702,7 +13702,7 @@
         <v>1</v>
       </c>
       <c r="C232" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.3">
@@ -13713,7 +13713,7 @@
         <v>2</v>
       </c>
       <c r="C233" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -13734,7 +13734,7 @@
         <v>266</v>
       </c>
       <c r="C1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -13745,7 +13745,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -13756,7 +13756,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -13767,7 +13767,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -13778,7 +13778,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -13789,7 +13789,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -13800,7 +13800,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -13811,7 +13811,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -13822,7 +13822,7 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -13833,7 +13833,7 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -13844,7 +13844,7 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -13855,7 +13855,7 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add triggers (PostgreSQL syntax) with UPDATE, DELETE, and INSERT tests
</commit_message>
<xml_diff>
--- a/sql/hotelchains.xlsx
+++ b/sql/hotelchains.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniela Bordeianu\Uni\CSI2132\room4u\sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C514FA6-EE96-4F5B-BDE3-2695A8ABA159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30654ABA-6F7F-43E9-A6CB-C2F4C36AD7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="1104" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="6" xr2:uid="{7AC72208-6A4A-45CD-80D5-6B3DF0A8B70B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="7" activeTab="10" xr2:uid="{7AC72208-6A4A-45CD-80D5-6B3DF0A8B70B}"/>
   </bookViews>
   <sheets>
     <sheet name="hotel_chain" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,7 @@
     <sheet name="processes" sheetId="23" r:id="rId23"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2116,7 +2117,7 @@
         <v>46170.541666666664</v>
       </c>
       <c r="D4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2130,7 +2131,7 @@
         <v>46218.416666666664</v>
       </c>
       <c r="D5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fix: update the schema for CASCADE/SET NULL on foreign keys to support trigger testing
</commit_message>
<xml_diff>
--- a/sql/hotelchains.xlsx
+++ b/sql/hotelchains.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniela Bordeianu\Uni\CSI2132\room4u\sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30654ABA-6F7F-43E9-A6CB-C2F4C36AD7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D3686A-C482-4C9C-BCA7-01922E0B283D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="7" activeTab="10" xr2:uid="{7AC72208-6A4A-45CD-80D5-6B3DF0A8B70B}"/>
+    <workbookView xWindow="2520" yWindow="1104" windowWidth="17280" windowHeight="9960" firstSheet="17" activeTab="21" xr2:uid="{7AC72208-6A4A-45CD-80D5-6B3DF0A8B70B}"/>
   </bookViews>
   <sheets>
     <sheet name="hotel_chain" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,6 @@
     <sheet name="processes" sheetId="23" r:id="rId23"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -59,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="407">
   <si>
     <t>chain_id</t>
   </si>
@@ -5361,7 +5360,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69DE4B2D-625D-427A-9E47-941A10C2C0DA}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -5397,24 +5396,36 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
-        <v>786124431</v>
+      <c r="A3">
+        <v>245667189</v>
       </c>
       <c r="B3" t="s">
+        <v>322</v>
+      </c>
+      <c r="C3">
+        <v>223761213</v>
+      </c>
+      <c r="D3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>111676789</v>
+      </c>
+      <c r="B4" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
-        <v>124567890</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4">
+        <v>223761213</v>
+      </c>
+      <c r="D4" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>245667189</v>
+        <v>222676789</v>
       </c>
       <c r="B5" t="s">
         <v>322</v>
@@ -5423,50 +5434,6 @@
         <v>223761213</v>
       </c>
       <c r="D5" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>662112345</v>
-      </c>
-      <c r="B6" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>223761213</v>
-      </c>
-      <c r="B7" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>111676789</v>
-      </c>
-      <c r="B8" t="s">
-        <v>323</v>
-      </c>
-      <c r="C8">
-        <v>223761213</v>
-      </c>
-      <c r="D8" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>222676789</v>
-      </c>
-      <c r="B9" t="s">
-        <v>322</v>
-      </c>
-      <c r="C9">
-        <v>223761213</v>
-      </c>
-      <c r="D9" t="s">
         <v>322</v>
       </c>
     </row>

</xml_diff>